<commit_message>
ajout xls pour imports
</commit_message>
<xml_diff>
--- a/export_pronos_v3.xlsx
+++ b/export_pronos_v3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d41a2cc4a867f612/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{680299BC-0E15-4DB6-94BD-AEDF46C29EAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{058F45A3-1FF4-4AF9-9BF4-B27FCD219EC2}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="8_{680299BC-0E15-4DB6-94BD-AEDF46C29EAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5D3505A7-8012-4FA1-A93F-73E5747B15D5}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3A54BC06-1FB7-4C75-9C7F-FEFDCAFB0ABF}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="636" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="606" uniqueCount="43">
   <si>
     <t>Antoine</t>
   </si>
@@ -160,9 +160,6 @@
   </si>
   <si>
     <t>Toulon</t>
-  </si>
-  <si>
-    <t>X</t>
   </si>
 </sst>
 </file>
@@ -526,7 +523,18 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2 4" xfId="1" xr:uid="{03DAA72D-66D2-4927-BE1B-DF974EB0FCA3}"/>
   </cellStyles>
-  <dxfs count="63">
+  <dxfs count="52">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FFFF0000"/>
@@ -557,6 +565,179 @@
       <fill>
         <patternFill patternType="none">
           <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF00B050"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -596,6 +777,7 @@
       <font>
         <b/>
         <i val="0"/>
+        <color rgb="FF00B050"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -605,11 +787,55 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
+        <color rgb="FFFF0000"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF00B050"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF00B050"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
         </patternFill>
       </fill>
     </dxf>
@@ -639,20 +865,11 @@
       <font>
         <b/>
         <i val="0"/>
+        <color rgb="FF00B050"/>
       </font>
       <fill>
         <patternFill patternType="none">
           <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -680,22 +897,23 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
-        <i val="0"/>
+        <color rgb="FFFF0000"/>
       </font>
       <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
+        <patternFill>
+          <bgColor theme="0"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF00B050"/>
       </font>
       <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
         </patternFill>
       </fill>
     </dxf>
@@ -723,280 +941,11 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FFFF0000"/>
       </font>
       <fill>
         <patternFill>
           <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF00B050"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF00B050"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF00B050"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF00B050"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF00B050"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF00B050"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1059,6 +1008,7 @@
       <font>
         <b/>
         <i val="0"/>
+        <color rgb="FF00B050"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -1090,52 +1040,22 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FFFF0000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <b/>
         <i val="0"/>
       </font>
       <fill>
         <patternFill patternType="none">
           <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1153,55 +1073,11 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FFFF0000"/>
       </font>
       <fill>
         <patternFill>
           <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF00B050"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1267,24 +1143,24 @@
       <sheetName val="export"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13"/>
-      <sheetData sheetId="14"/>
-      <sheetData sheetId="15"/>
-      <sheetData sheetId="16"/>
-      <sheetData sheetId="17"/>
+      <sheetData sheetId="0" refreshError="1"/>
+      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="2" refreshError="1"/>
+      <sheetData sheetId="3" refreshError="1"/>
+      <sheetData sheetId="4" refreshError="1"/>
+      <sheetData sheetId="5" refreshError="1"/>
+      <sheetData sheetId="6" refreshError="1"/>
+      <sheetData sheetId="7" refreshError="1"/>
+      <sheetData sheetId="8" refreshError="1"/>
+      <sheetData sheetId="9" refreshError="1"/>
+      <sheetData sheetId="10" refreshError="1"/>
+      <sheetData sheetId="11" refreshError="1"/>
+      <sheetData sheetId="12" refreshError="1"/>
+      <sheetData sheetId="13" refreshError="1"/>
+      <sheetData sheetId="14" refreshError="1"/>
+      <sheetData sheetId="15" refreshError="1"/>
+      <sheetData sheetId="16" refreshError="1"/>
+      <sheetData sheetId="17" refreshError="1"/>
       <sheetData sheetId="18">
         <row r="21">
           <cell r="T21">
@@ -1335,27 +1211,27 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="19"/>
-      <sheetData sheetId="20"/>
-      <sheetData sheetId="21"/>
-      <sheetData sheetId="22"/>
-      <sheetData sheetId="23"/>
-      <sheetData sheetId="24"/>
-      <sheetData sheetId="25"/>
-      <sheetData sheetId="26"/>
-      <sheetData sheetId="27"/>
-      <sheetData sheetId="28"/>
-      <sheetData sheetId="29"/>
-      <sheetData sheetId="30"/>
-      <sheetData sheetId="31"/>
-      <sheetData sheetId="32"/>
-      <sheetData sheetId="33"/>
-      <sheetData sheetId="34"/>
-      <sheetData sheetId="35"/>
-      <sheetData sheetId="36"/>
-      <sheetData sheetId="37"/>
-      <sheetData sheetId="38"/>
-      <sheetData sheetId="39"/>
+      <sheetData sheetId="19" refreshError="1"/>
+      <sheetData sheetId="20" refreshError="1"/>
+      <sheetData sheetId="21" refreshError="1"/>
+      <sheetData sheetId="22" refreshError="1"/>
+      <sheetData sheetId="23" refreshError="1"/>
+      <sheetData sheetId="24" refreshError="1"/>
+      <sheetData sheetId="25" refreshError="1"/>
+      <sheetData sheetId="26" refreshError="1"/>
+      <sheetData sheetId="27" refreshError="1"/>
+      <sheetData sheetId="28" refreshError="1"/>
+      <sheetData sheetId="29" refreshError="1"/>
+      <sheetData sheetId="30" refreshError="1"/>
+      <sheetData sheetId="31" refreshError="1"/>
+      <sheetData sheetId="32" refreshError="1"/>
+      <sheetData sheetId="33" refreshError="1"/>
+      <sheetData sheetId="34" refreshError="1"/>
+      <sheetData sheetId="35" refreshError="1"/>
+      <sheetData sheetId="36" refreshError="1"/>
+      <sheetData sheetId="37" refreshError="1"/>
+      <sheetData sheetId="38" refreshError="1"/>
+      <sheetData sheetId="39" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -1858,8 +1734,8 @@
       <c r="F7" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="G7" s="3" t="s">
-        <v>43</v>
+      <c r="G7" s="3">
+        <v>1</v>
       </c>
       <c r="H7" s="11">
         <v>47</v>
@@ -1914,8 +1790,8 @@
       <c r="F9" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="G9" s="9" t="s">
-        <v>43</v>
+      <c r="G9" s="9">
+        <v>1</v>
       </c>
       <c r="H9" s="4">
         <f>'[1]T (16)'!T21</f>
@@ -2006,8 +1882,8 @@
       <c r="F12" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="G12" s="3" t="s">
-        <v>43</v>
+      <c r="G12" s="3">
+        <v>1</v>
       </c>
       <c r="H12" s="4">
         <f>'[1]T (16)'!T24</f>
@@ -2047,8 +1923,8 @@
         <f>'[1]T (16)'!V25</f>
         <v>35</v>
       </c>
-      <c r="J13" s="17" t="s">
-        <v>43</v>
+      <c r="J13" s="17">
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
@@ -2070,8 +1946,8 @@
       <c r="F14" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="G14" s="3" t="s">
-        <v>43</v>
+      <c r="G14" s="3">
+        <v>1</v>
       </c>
       <c r="H14" s="4">
         <f>'[1]T (16)'!T26</f>
@@ -2160,8 +2036,8 @@
       <c r="F17" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="G17" s="3" t="s">
-        <v>43</v>
+      <c r="G17" s="3">
+        <v>1</v>
       </c>
       <c r="H17" s="11">
         <v>32</v>
@@ -2253,8 +2129,8 @@
       <c r="I20" s="14">
         <v>52</v>
       </c>
-      <c r="J20" s="17" t="s">
-        <v>43</v>
+      <c r="J20" s="17">
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
@@ -2276,8 +2152,8 @@
       <c r="F21" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="G21" s="3" t="s">
-        <v>43</v>
+      <c r="G21" s="3">
+        <v>1</v>
       </c>
       <c r="H21" s="11">
         <v>38</v>
@@ -2306,8 +2182,8 @@
       <c r="F22" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="G22" s="5" t="s">
-        <v>43</v>
+      <c r="G22" s="5">
+        <v>1</v>
       </c>
       <c r="H22" s="12">
         <v>28</v>
@@ -2444,8 +2320,8 @@
       <c r="F28" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="G28" s="3" t="s">
-        <v>43</v>
+      <c r="G28" s="3">
+        <v>1</v>
       </c>
       <c r="H28" s="11">
         <v>53</v>
@@ -2474,8 +2350,8 @@
       <c r="F29" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="G29" s="5" t="s">
-        <v>43</v>
+      <c r="G29" s="5">
+        <v>1</v>
       </c>
       <c r="H29" s="12">
         <v>43</v>
@@ -2952,8 +2828,8 @@
       <c r="F46" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="G46" s="3" t="s">
-        <v>43</v>
+      <c r="G46" s="3">
+        <v>1</v>
       </c>
       <c r="H46" s="11">
         <v>44</v>
@@ -3038,8 +2914,8 @@
       <c r="F49" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="G49" s="3" t="s">
-        <v>43</v>
+      <c r="G49" s="3">
+        <v>1</v>
       </c>
       <c r="H49" s="11">
         <v>43</v>
@@ -3320,8 +3196,8 @@
       <c r="F59" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="G59" s="3" t="s">
-        <v>43</v>
+      <c r="G59" s="3">
+        <v>1</v>
       </c>
       <c r="H59" s="11">
         <v>32</v>
@@ -3434,8 +3310,8 @@
       <c r="F63" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="G63" s="3" t="s">
-        <v>43</v>
+      <c r="G63" s="3">
+        <v>1</v>
       </c>
       <c r="H63" s="11">
         <v>35</v>
@@ -3884,8 +3760,8 @@
       <c r="F79" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="G79" s="9" t="s">
-        <v>43</v>
+      <c r="G79" s="9">
+        <v>1</v>
       </c>
       <c r="H79" s="10">
         <v>47</v>
@@ -3942,8 +3818,8 @@
       <c r="F81" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="G81" s="3" t="s">
-        <v>43</v>
+      <c r="G81" s="3">
+        <v>1</v>
       </c>
       <c r="H81" s="11">
         <v>47</v>
@@ -3972,8 +3848,8 @@
       <c r="F82" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="G82" s="3" t="s">
-        <v>43</v>
+      <c r="G82" s="3">
+        <v>1</v>
       </c>
       <c r="H82" s="11">
         <v>47</v>
@@ -4002,8 +3878,8 @@
       <c r="F83" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="G83" s="3" t="s">
-        <v>43</v>
+      <c r="G83" s="3">
+        <v>1</v>
       </c>
       <c r="H83" s="11">
         <v>47</v>
@@ -4032,8 +3908,8 @@
       <c r="F84" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="G84" s="3" t="s">
-        <v>43</v>
+      <c r="G84" s="3">
+        <v>1</v>
       </c>
       <c r="H84" s="11">
         <v>47</v>
@@ -4230,8 +4106,8 @@
       <c r="F91" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="G91" s="3" t="s">
-        <v>43</v>
+      <c r="G91" s="3">
+        <v>1</v>
       </c>
       <c r="H91" s="11">
         <v>32</v>
@@ -4407,8 +4283,8 @@
       <c r="I97" s="14">
         <v>43</v>
       </c>
-      <c r="J97" s="17" t="s">
-        <v>43</v>
+      <c r="J97" s="17">
+        <v>1</v>
       </c>
     </row>
     <row r="98" spans="1:10" x14ac:dyDescent="0.3">
@@ -4430,8 +4306,8 @@
       <c r="F98" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="G98" s="3" t="s">
-        <v>43</v>
+      <c r="G98" s="3">
+        <v>1</v>
       </c>
       <c r="H98" s="11">
         <v>34</v>
@@ -4628,8 +4504,8 @@
       <c r="F105" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="G105" s="3" t="s">
-        <v>43</v>
+      <c r="G105" s="3">
+        <v>1</v>
       </c>
       <c r="H105" s="11">
         <v>39</v>
@@ -4714,8 +4590,8 @@
       <c r="F108" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="G108" s="3" t="s">
-        <v>43</v>
+      <c r="G108" s="3">
+        <v>1</v>
       </c>
       <c r="H108" s="11">
         <v>39</v>
@@ -4744,8 +4620,8 @@
       <c r="F109" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="G109" s="3" t="s">
-        <v>43</v>
+      <c r="G109" s="3">
+        <v>1</v>
       </c>
       <c r="H109" s="11">
         <v>31</v>
@@ -4809,8 +4685,8 @@
       <c r="I111" s="14">
         <v>32</v>
       </c>
-      <c r="J111" s="17" t="s">
-        <v>43</v>
+      <c r="J111" s="17">
+        <v>1</v>
       </c>
     </row>
     <row r="112" spans="1:10" x14ac:dyDescent="0.3">
@@ -4832,8 +4708,8 @@
       <c r="F112" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="G112" s="3" t="s">
-        <v>43</v>
+      <c r="G112" s="3">
+        <v>1</v>
       </c>
       <c r="H112" s="11">
         <v>48</v>
@@ -4862,8 +4738,8 @@
       <c r="F113" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="G113" s="5" t="s">
-        <v>43</v>
+      <c r="G113" s="5">
+        <v>1</v>
       </c>
       <c r="H113" s="12">
         <v>34</v>
@@ -4920,7 +4796,9 @@
       <c r="F115" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="G115" s="3"/>
+      <c r="G115" s="3">
+        <v>1</v>
+      </c>
       <c r="H115" s="11">
         <v>33</v>
       </c>
@@ -4948,7 +4826,9 @@
       <c r="F116" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="G116" s="3"/>
+      <c r="G116" s="3">
+        <v>1</v>
+      </c>
       <c r="H116" s="11">
         <v>41</v>
       </c>
@@ -4976,7 +4856,9 @@
       <c r="F117" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="G117" s="3"/>
+      <c r="G117" s="3">
+        <v>1</v>
+      </c>
       <c r="H117" s="11">
         <v>32</v>
       </c>
@@ -5011,8 +4893,8 @@
       <c r="I118" s="14">
         <v>37</v>
       </c>
-      <c r="J118" s="17" t="s">
-        <v>43</v>
+      <c r="J118" s="17">
+        <v>1</v>
       </c>
     </row>
     <row r="119" spans="1:10" x14ac:dyDescent="0.3">
@@ -12543,207 +12425,176 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G7 H9:I15 G16:G21 G23 G30:G35 G51:G56">
-    <cfRule type="cellIs" dxfId="62" priority="112" operator="lessThan">
-      <formula>1</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="61" priority="113" operator="equal">
+  <conditionalFormatting sqref="G2:G7 H9:I15 G23 G30:G35 G51:G56">
+    <cfRule type="cellIs" dxfId="51" priority="114" operator="notEqual">
       <formula>$E2</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="60" priority="114" operator="notEqual">
+    <cfRule type="cellIs" dxfId="50" priority="113" operator="equal">
       <formula>$E2</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="G2:G23">
+    <cfRule type="cellIs" dxfId="49" priority="108" operator="lessThan">
+      <formula>1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G8 G22 G29 G57:G63">
+    <cfRule type="cellIs" dxfId="48" priority="123" operator="notEqual">
+      <formula>$E13</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="47" priority="122" operator="equal">
+      <formula>$E13</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G9:G21">
+    <cfRule type="cellIs" dxfId="46" priority="110" operator="notEqual">
+      <formula>$E9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="45" priority="109" operator="equal">
+      <formula>$E9</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G28">
+    <cfRule type="cellIs" dxfId="44" priority="148" operator="equal">
+      <formula>$E28</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="43" priority="149" operator="notEqual">
+      <formula>$E28</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G28:G120">
+    <cfRule type="cellIs" dxfId="42" priority="4" operator="lessThan">
+      <formula>1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G36:G42">
+    <cfRule type="cellIs" dxfId="41" priority="157" operator="equal">
+      <formula>$E41</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="40" priority="158" operator="notEqual">
+      <formula>$E41</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G43:G49 G64:G70">
+    <cfRule type="cellIs" dxfId="39" priority="142" operator="notEqual">
+      <formula>$E53</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="38" priority="141" operator="equal">
+      <formula>$E53</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G50 G71:G77">
+    <cfRule type="cellIs" dxfId="37" priority="134" operator="notEqual">
+      <formula>$E65</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="36" priority="133" operator="equal">
+      <formula>$E65</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G78:G84">
+    <cfRule type="cellIs" dxfId="35" priority="30" operator="notEqual">
+      <formula>$E98</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="34" priority="29" operator="equal">
+      <formula>$E98</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G85:G91">
+    <cfRule type="cellIs" dxfId="33" priority="22" operator="notEqual">
+      <formula>$E110</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="32" priority="21" operator="equal">
+      <formula>$E110</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G92:G98">
+    <cfRule type="cellIs" dxfId="31" priority="13" operator="equal">
+      <formula>$E122</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="30" priority="14" operator="notEqual">
+      <formula>$E122</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G99:G105">
+    <cfRule type="cellIs" dxfId="29" priority="5" operator="equal">
+      <formula>$E134</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="28" priority="6" operator="notEqual">
+      <formula>$E134</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G106:G112">
+    <cfRule type="cellIs" dxfId="27" priority="168" operator="notEqual">
+      <formula>$E146</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="26" priority="167" operator="equal">
+      <formula>$E146</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G113:G119">
+    <cfRule type="cellIs" dxfId="25" priority="184" operator="notEqual">
+      <formula>$E158</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="24" priority="183" operator="equal">
+      <formula>$E158</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G120">
+    <cfRule type="cellIs" dxfId="23" priority="199" operator="equal">
+      <formula>$E170</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="22" priority="200" operator="notEqual">
+      <formula>$E170</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="H2:H7 H16:H21 H23 H30:H35 H51:H56">
-    <cfRule type="cellIs" dxfId="59" priority="115" operator="equal">
+    <cfRule type="cellIs" dxfId="21" priority="115" operator="equal">
       <formula>$F2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G8 G22 G29 G57:G63">
-    <cfRule type="cellIs" dxfId="58" priority="121" operator="lessThan">
-      <formula>1</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="57" priority="122" operator="equal">
-      <formula>$E13</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="56" priority="123" operator="notEqual">
-      <formula>$E13</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="H8 H22 H29 H57:H63">
-    <cfRule type="cellIs" dxfId="55" priority="125" operator="equal">
+    <cfRule type="cellIs" dxfId="20" priority="125" operator="equal">
       <formula>$F13</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I7 I16:I23 I28:I120">
-    <cfRule type="cellIs" dxfId="54" priority="111" operator="equal">
-      <formula>$H2</formula>
+  <conditionalFormatting sqref="H28">
+    <cfRule type="cellIs" dxfId="19" priority="154" operator="equal">
+      <formula>$F28</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I8">
-    <cfRule type="cellIs" dxfId="53" priority="127" operator="equal">
-      <formula>$H13</formula>
+  <conditionalFormatting sqref="H36:H42">
+    <cfRule type="cellIs" dxfId="18" priority="162" operator="equal">
+      <formula>$F41</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G9:G15">
-    <cfRule type="cellIs" dxfId="52" priority="108" operator="lessThan">
-      <formula>1</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="51" priority="109" operator="equal">
-      <formula>$E9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="50" priority="110" operator="notEqual">
-      <formula>$E9</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J9:J15">
-    <cfRule type="cellIs" dxfId="49" priority="105" operator="lessThan">
-      <formula>1</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="48" priority="106" operator="equal">
-      <formula>$I9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="47" priority="107" operator="notEqual">
-      <formula>$I9</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G50 G71:G77">
-    <cfRule type="cellIs" dxfId="46" priority="132" operator="lessThan">
-      <formula>1</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="45" priority="133" operator="equal">
-      <formula>$E65</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="44" priority="134" operator="notEqual">
-      <formula>$E65</formula>
+  <conditionalFormatting sqref="H43:H49 H64:H70">
+    <cfRule type="cellIs" dxfId="17" priority="143" operator="equal">
+      <formula>$F53</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H50 H71:H77">
-    <cfRule type="cellIs" dxfId="43" priority="135" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="135" operator="equal">
       <formula>$F65</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G43:G49 G64:G70">
-    <cfRule type="cellIs" dxfId="42" priority="140" operator="lessThan">
-      <formula>1</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="41" priority="141" operator="equal">
-      <formula>$E53</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="40" priority="142" operator="notEqual">
-      <formula>$E53</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H43:H49 H64:H70">
-    <cfRule type="cellIs" dxfId="39" priority="143" operator="equal">
-      <formula>$F53</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G28">
-    <cfRule type="cellIs" dxfId="38" priority="147" operator="lessThan">
-      <formula>1</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="37" priority="148" operator="equal">
-      <formula>$E28</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="36" priority="149" operator="notEqual">
-      <formula>$E28</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H28">
-    <cfRule type="cellIs" dxfId="35" priority="154" operator="equal">
-      <formula>$F28</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G36:G42">
-    <cfRule type="cellIs" dxfId="34" priority="156" operator="lessThan">
-      <formula>1</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="33" priority="157" operator="equal">
-      <formula>$E41</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="32" priority="158" operator="notEqual">
-      <formula>$E41</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H36:H42">
-    <cfRule type="cellIs" dxfId="31" priority="162" operator="equal">
-      <formula>$F41</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G78:G84">
-    <cfRule type="cellIs" dxfId="30" priority="28" operator="lessThan">
-      <formula>1</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="29" priority="29" operator="equal">
-      <formula>$E98</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="30" operator="notEqual">
-      <formula>$E98</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="H78:H84">
-    <cfRule type="cellIs" dxfId="27" priority="32" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="32" operator="equal">
       <formula>$F98</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G85:G91">
-    <cfRule type="cellIs" dxfId="26" priority="20" operator="lessThan">
-      <formula>1</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="21" operator="equal">
-      <formula>$E110</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="22" operator="notEqual">
-      <formula>$E110</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="H85:H91">
-    <cfRule type="cellIs" dxfId="23" priority="24" operator="equal">
+    <cfRule type="cellIs" dxfId="14" priority="24" operator="equal">
       <formula>$F110</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G92:G98">
-    <cfRule type="cellIs" dxfId="22" priority="12" operator="lessThan">
-      <formula>1</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="13" operator="equal">
-      <formula>$E122</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="20" priority="14" operator="notEqual">
-      <formula>$E122</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="H92:H98">
-    <cfRule type="cellIs" dxfId="19" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="16" operator="equal">
       <formula>$F122</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G99:G105">
-    <cfRule type="cellIs" dxfId="18" priority="4" operator="lessThan">
-      <formula>1</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="17" priority="5" operator="equal">
-      <formula>$E134</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="6" operator="notEqual">
-      <formula>$E134</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="H99:H105">
-    <cfRule type="cellIs" dxfId="15" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="8" operator="equal">
       <formula>$F134</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G106:G112">
-    <cfRule type="cellIs" dxfId="14" priority="166" operator="lessThan">
-      <formula>1</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="167" operator="equal">
-      <formula>$E146</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="168" operator="notEqual">
-      <formula>$E146</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H106:H112">
@@ -12751,47 +12602,55 @@
       <formula>$F146</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G113:G119">
-    <cfRule type="cellIs" dxfId="10" priority="182" operator="lessThan">
-      <formula>1</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="183" operator="equal">
-      <formula>$E158</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="184" operator="notEqual">
-      <formula>$E158</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="H113:H119">
-    <cfRule type="cellIs" dxfId="7" priority="186" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="186" operator="equal">
       <formula>$F158</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G120">
-    <cfRule type="cellIs" dxfId="6" priority="198" operator="lessThan">
-      <formula>1</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="199" operator="equal">
-      <formula>$E170</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="200" operator="notEqual">
-      <formula>$E170</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="H120">
-    <cfRule type="cellIs" dxfId="3" priority="202" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="202" operator="equal">
       <formula>$F170</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J28:J120 J16:J23">
-    <cfRule type="cellIs" dxfId="2" priority="203" operator="lessThan">
+  <conditionalFormatting sqref="H9:I15">
+    <cfRule type="cellIs" dxfId="8" priority="112" operator="lessThan">
       <formula>1</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="204" operator="equal">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I2:I7 I16:I23 I28:I120">
+    <cfRule type="cellIs" dxfId="7" priority="111" operator="equal">
+      <formula>$H2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I8">
+    <cfRule type="cellIs" dxfId="6" priority="127" operator="equal">
+      <formula>$H13</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J9:J15">
+    <cfRule type="cellIs" dxfId="5" priority="107" operator="notEqual">
+      <formula>$I9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="106" operator="equal">
+      <formula>$I9</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J9:J23">
+    <cfRule type="cellIs" dxfId="3" priority="105" operator="lessThan">
+      <formula>1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J16:J23 J28:J120">
+    <cfRule type="cellIs" dxfId="2" priority="204" operator="equal">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="205" operator="notEqual">
+    <cfRule type="cellIs" dxfId="1" priority="205" operator="notEqual">
       <formula>#REF!</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J28:J120">
+    <cfRule type="cellIs" dxfId="0" priority="203" operator="lessThan">
+      <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>